<commit_message>
up Inom added to TOKZ
</commit_message>
<xml_diff>
--- a/mode_docx_gen/pmi_tokz/torpn_modes/ТО РПН_1.xlsx
+++ b/mode_docx_gen/pmi_tokz/torpn_modes/ТО РПН_1.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SGF_Parameters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outputs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -455,17 +456,6 @@
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,135 +471,80 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>T1_ptoc1_lvtoc</t>
+          <t>SGF1_hvptoc1_lovctoc</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Iset_ptoc1_lvtoc</t>
+          <t>SGF1_ptoc1_lvarctoc</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>SGF1_hvptoc1_lovctoc</t>
+          <t>SGF2_ptoc1_lvarctoc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>T1_hvptoc1_lovctoc</t>
+          <t>SGF1_ptoc1_ltcblktoc</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Iset_hvptoc1_lovctoc</t>
+          <t>SGF1_nsptoc1_lvnstoc</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>SGF1_ptoc1_lvarctoc</t>
+          <t>SGF2_nsptoc1_lvnstoc</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>SGF2_ptoc1_lvarctoc</t>
+          <t>SGF1_ptrc1_ttoclgc</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Iset_ptoc1_lvarctoc</t>
+          <t>SGF2_ptrc1_ttoclgc</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>SGF1_ptoc1_ltcblktoc</t>
+          <t>SGF3_ptrc1_ttoclgc</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Iset_ptoc1_ltcblktoc</t>
+          <t>SGF1_ptrc1_tofflvlgc</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>SGF1_nsptoc1_lvnstoc</t>
+          <t>SGF1_rbre1_tofflvlgc</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>SGF2_nsptoc1_lvnstoc</t>
+          <t>SGF2_rbre1_tofflvlgc</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>T1_nsptoc1_lvnstoc</t>
+          <t>SGF3_rbre1_tofflvlgc</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>I2set_nsptoc1_lvnstoc</t>
+          <t>SGF1_rblc1_tofflvlgc</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>RatioSet_nsptoc1_lvnstoc</t>
+          <t>SGF2_rblc1_tofflvlgc</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>In_nsptoc1_lvnstoc</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptrc1_ttoclgc</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>SGF2_ptrc1_ttoclgc</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>SGF3_ptrc1_ttoclgc</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>T1_ptrc1_ttoclgc</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_ptrc1_tofflvlgc</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_rbre1_tofflvlgc</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>SGF2_rbre1_tofflvlgc</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>SGF3_rbre1_tofflvlgc</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>SGF1_rblc1_tofflvlgc</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>SGF2_rblc1_tofflvlgc</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>SGF3_rblc1_tofflvlgc</t>
         </is>
@@ -622,11 +557,11 @@
       <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -634,8 +569,8 @@
       <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
+      <c r="G2" t="n">
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -643,64 +578,31 @@
       <c r="I2" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>1</v>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M2" t="n">
-        <v>0</v>
+      <c r="M2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="2" t="n">
-        <v>1</v>
+      <c r="O2" t="n">
+        <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="Q2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="W2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" t="n">
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -710,6 +612,125 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>T1_ptoc1_lvtoc</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Iset_ptoc1_lvtoc</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>T1_hvptoc1_lovctoc</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Iset_hvptoc1_lovctoc</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Iset_ptoc1_lvarctoc</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Iset_ptoc1_ltcblktoc</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>T1_nsptoc1_lvnstoc</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>I2set_nsptoc1_lvnstoc</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>RatioSet_nsptoc1_lvnstoc</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>In_nsptoc1_lvnstoc</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>T1_ptrc1_ttoclgc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -954,7 +975,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>